<commit_message>
Assignments of 10th July
</commit_message>
<xml_diff>
--- a/9th_of_July/AzureDevOps_Epic1_Feature1_TestCase.xlsx
+++ b/9th_of_July/AzureDevOps_Epic1_Feature1_TestCase.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gargd\Desktop\Test\MyAssignmentsRepo\8th_of_July\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gargd\Desktop\Test\MyAssignmentsRepo\9th_of_July\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{921E2A6C-0B10-4C78-8B04-17256DA07A5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81E2F5BE-B603-4386-B772-0210E0B1293D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="348" yWindow="720" windowWidth="21600" windowHeight="11100" xr2:uid="{2CC64075-47C3-4778-8FB5-A23C612AEB7E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2CC64075-47C3-4778-8FB5-A23C612AEB7E}"/>
   </bookViews>
   <sheets>
     <sheet name="AzureDevOps_Epic41_Feature1_TC" sheetId="1" r:id="rId1"/>
@@ -1079,14 +1079,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1178,49 +1171,49 @@
   </cellStyleXfs>
   <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>

</xml_diff>